<commit_message>
Added entry for Kelsey Bryant
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H179"/>
+  <dimension ref="A1:H180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6062,10 +6062,8 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t xml:space="preserve">333 </t>
-        </is>
+      <c r="A179" t="n">
+        <v>333</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -6096,6 +6094,40 @@
       <c r="H179" t="inlineStr">
         <is>
           <t>Seth Charley</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">329 </t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Kelsey Bryant</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D180" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E180" s="1" t="n">
+        <v>46360.99930555555</v>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>329 - Chevy Trail Boss, White</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Kelsey Bryant</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Anita Joy Antoninka
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H180"/>
+  <dimension ref="A1:H181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6098,10 +6098,8 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t xml:space="preserve">329 </t>
-        </is>
+      <c r="A180" t="n">
+        <v>329</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -6128,6 +6126,44 @@
       <c r="H180" t="inlineStr">
         <is>
           <t>Kelsey Bryant</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">333 </t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Anita Joy Antoninka</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D181" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E181" s="1" t="n">
+        <v>46289.99930555555</v>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>field work at north rim of gc. no dirt roads, just space for gear and people</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Seth Charley</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated data via interactive editor
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H181"/>
+  <dimension ref="A1:H180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5999,11 +5999,11 @@
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>268</v>
+        <v>332</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>OUT OF COMMISSION</t>
+          <t>Salli Dymond</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -6012,30 +6012,30 @@
         </is>
       </c>
       <c r="D177" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="E177" s="1" t="n">
         <v>46276.99930555555</v>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>268 - 2017 Ford F-150, Silver(6 Seats)</t>
-        </is>
-      </c>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>Needs oil change asap</t>
-        </is>
-      </c>
-      <c r="H177" t="inlineStr"/>
+          <t>332 - 2009 Dodge Dakota, White (5 Seats)</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Cody Folk</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Salli Dymond</t>
+          <t>Anita Joy Antoninka</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -6044,30 +6044,34 @@
         </is>
       </c>
       <c r="D178" s="1" t="n">
-        <v>46274</v>
+        <v>46280</v>
       </c>
       <c r="E178" s="1" t="n">
-        <v>46276.99930555555</v>
+        <v>46289.99930555555</v>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>332 - 2009 Dodge Dakota, White (5 Seats)</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr"/>
+          <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>field work at north rim of gc. no dirt roads, just space for gear and people</t>
+        </is>
+      </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Cody Folk</t>
+          <t>Seth Charley</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Anita Joy Antoninka</t>
+          <t>Kelsey Bryant</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -6076,34 +6080,30 @@
         </is>
       </c>
       <c r="D179" s="1" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="E179" s="1" t="n">
-        <v>46289.99930555555</v>
+        <v>46360.99930555555</v>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
-        </is>
-      </c>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>field work at north rim of gc. no dirt roads, just space for gear and people</t>
-        </is>
-      </c>
+          <t>329 - Chevy Trail Boss, White</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Seth Charley</t>
+          <t>Kelsey Bryant</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Kelsey Bryant</t>
+          <t>Anita Joy Antoninka</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -6112,56 +6112,22 @@
         </is>
       </c>
       <c r="D180" s="1" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E180" s="1" t="n">
-        <v>46360.99930555555</v>
+        <v>46289.99930555555</v>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>329 - Chevy Trail Boss, White</t>
-        </is>
-      </c>
-      <c r="G180" t="inlineStr"/>
+          <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>field work at north rim of gc. no dirt roads, just space for gear and people</t>
+        </is>
+      </c>
       <c r="H180" t="inlineStr">
-        <is>
-          <t>Kelsey Bryant</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t xml:space="preserve">333 </t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>Anita Joy Antoninka</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="D181" s="1" t="n">
-        <v>46280</v>
-      </c>
-      <c r="E181" s="1" t="n">
-        <v>46289.99930555555</v>
-      </c>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
-        </is>
-      </c>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>field work at north rim of gc. no dirt roads, just space for gear and people</t>
-        </is>
-      </c>
-      <c r="H181" t="inlineStr">
         <is>
           <t>Seth Charley</t>
         </is>

</xml_diff>

<commit_message>
Added entry for OUT OF COMMISSION
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H181"/>
+  <dimension ref="A1:H182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6134,10 +6134,8 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t xml:space="preserve">321 </t>
-        </is>
+      <c r="A181" t="n">
+        <v>321</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -6166,6 +6164,40 @@
           <t>Mariola Barerra</t>
         </is>
       </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330 </t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>OUT OF COMMISSION</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D182" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E182" s="1" t="n">
+        <v>46285.99930555555</v>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>330 - Toyota Camry</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Getting Bumper Fixed</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added entry for Kristen Waring
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H182"/>
+  <dimension ref="A1:H183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6166,10 +6166,8 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t xml:space="preserve">330 </t>
-        </is>
+      <c r="A182" t="n">
+        <v>330</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -6198,6 +6196,40 @@
         </is>
       </c>
       <c r="H182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">333 </t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Kristen Waring</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="D183" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E183" s="1" t="n">
+        <v>46290.99930555555</v>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>333 - 2017 Toyota Tacoma, Charcoal (5 Seats)</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Abirel Acharya</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added entry for Jill Beckmann
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6198,10 +6198,8 @@
       <c r="H182" t="inlineStr"/>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t xml:space="preserve">268 </t>
-        </is>
+      <c r="A183" t="n">
+        <v>268</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -6228,6 +6226,44 @@
       <c r="H183" t="inlineStr">
         <is>
           <t>Abirel Acharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">321 </t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Jill Beckmann</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D184" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E184" s="1" t="n">
+        <v>46290.99930555555</v>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>321 - Chevy Trail Boss, White</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>FOR 211 on Thursday - will drive 2 miles; Provost Visit on Friday - will drive to Centennial Forest ~ 30 miles</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Jill Beckmann, Villette Barlow</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Matthew Bowker
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6230,10 +6230,8 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t xml:space="preserve">321 </t>
-        </is>
+      <c r="A184" t="n">
+        <v>321</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -6264,6 +6262,44 @@
       <c r="H184" t="inlineStr">
         <is>
           <t>Jill Beckmann, Villette Barlow</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330 </t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Matthew Bowker</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D185" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E185" s="1" t="n">
+        <v>46326.99930555555</v>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>330 - Toyota Camry</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I will be in town to arrange CrustNet-related field work and to make one trip to Moab, UT to drop off equipment and samples. I will request separate trucks for the field work, so this request is just for my in-town work responsibilities AND the trip to Moab, UT. My return date for the vehicle is likely 10/28, but I put the end of the month here just in case something comes up and the trip home is delayed. </t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Sierra Gugel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Georgia Roberts
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6410,10 +6410,8 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">333 </t>
-        </is>
+      <c r="A189" t="n">
+        <v>333</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -6440,6 +6438,40 @@
       <c r="H189" t="inlineStr">
         <is>
           <t>Seth Charley</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330 </t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Georgia Roberts</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D190" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E190" s="1" t="n">
+        <v>46295.99930555555</v>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>330 - Toyota Camry</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Caelin Dicke</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Salli Dymond
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6538,10 +6538,8 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>331</t>
-        </is>
+      <c r="A193" t="n">
+        <v>331</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -6568,6 +6566,40 @@
       <c r="H193" t="inlineStr">
         <is>
           <t>Anita Antoninka</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330 </t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Salli Dymond</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D194" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E194" s="1" t="n">
+        <v>46304.99930555555</v>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>330 - Toyota Camry</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Cody Folk</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added entry for Seafha Ramos
</commit_message>
<xml_diff>
--- a/Vehicle_Checkout_List.xlsx
+++ b/Vehicle_Checkout_List.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H207"/>
+  <dimension ref="A1:H208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6986,10 +6986,8 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t xml:space="preserve">330 </t>
-        </is>
+      <c r="A207" t="n">
+        <v>330</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -7016,6 +7014,40 @@
       <c r="H207" t="inlineStr">
         <is>
           <t>Caelin Dicke</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330 </t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Seafha Ramos</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="D208" s="1" t="n">
+        <v>46331</v>
+      </c>
+      <c r="E208" s="1" t="n">
+        <v>46350.99930555555</v>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>330 - Toyota Camry</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr"/>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Seafha Ramos</t>
         </is>
       </c>
     </row>

</xml_diff>